<commit_message>
Fill out stack spreadsheet story points
</commit_message>
<xml_diff>
--- a/documentation/stack spreadsheet.xlsx
+++ b/documentation/stack spreadsheet.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+  <si>
+    <t xml:space="preserve">Requirement ID</t>
+  </si>
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -34,6 +37,9 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
+    <t xml:space="preserve">Sprint No.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total Items:</t>
   </si>
   <si>
@@ -52,16 +58,22 @@
     <t xml:space="preserve">Detect mouse movements to indicate swapping tiles</t>
   </si>
   <si>
+    <t xml:space="preserve">Sprints:</t>
+  </si>
+  <si>
     <t xml:space="preserve">Swapping Tiles</t>
   </si>
   <si>
     <t xml:space="preserve">Functionality to move/swap tiles</t>
   </si>
   <si>
+    <t xml:space="preserve">Story Points/Sprint:</t>
+  </si>
+  <si>
     <t xml:space="preserve">Detecting Matches</t>
   </si>
   <si>
-    <t xml:space="preserve">Detecting matches in a general sense</t>
+    <t xml:space="preserve">Detecting matches in a general sense (detecting every tile involved in tile in the match)</t>
   </si>
   <si>
     <t xml:space="preserve">Tile Clearing Mechanic</t>
@@ -91,7 +103,7 @@
     <t xml:space="preserve">Powerup creation</t>
   </si>
   <si>
-    <t xml:space="preserve">Create powerup after a special match</t>
+    <t xml:space="preserve">Create powerup after a special match (i.e. the powerup tile itself on the board)</t>
   </si>
   <si>
     <t xml:space="preserve">Powerups</t>
@@ -197,7 +209,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,13 +232,26 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A6099"/>
+        <bgColor rgb="FF666699"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -263,8 +288,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -277,7 +306,15 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2A6099"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -293,7 +330,75 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF2A6099"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -474,316 +579,487 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="83.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="86.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.98"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="0" t="s">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="0" t="n">
-        <f aca="false">COUNTA(A2:A10000)</f>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="n">
+        <f aca="false">COUNTA(B2:B10000)</f>
         <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="B2" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="0" t="n">
+        <f aca="false">SUM(D:D)</f>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="F2" s="0" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <f aca="false">I2/I3</f>
+        <v>12.6666666666667</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="G2" s="0" t="n">
-        <f aca="false">SUM(C:C)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="B8" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B9" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E12" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="0" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="D24" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B11" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="0" t="s">
+      <c r="B25" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B22" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="0" t="n">
+      <c r="B26" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="D24" s="0" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>55</v>
+      <c r="D26" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>